<commit_message>
Auto backup 2026-07-02 09:35:02
</commit_message>
<xml_diff>
--- a/SwissTechShehzad/jbl speaker.xlsx
+++ b/SwissTechShehzad/jbl speaker.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{36B1C085-ABF2-4461-AC8F-8D1D86E156E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F325888-0465-4D76-92BA-6C55E724EE8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C2E5228D-3AF2-4BEA-A542-C58324084CB1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -135,13 +136,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -480,27 +487,27 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="3">
-        <v>299</v>
+      <c r="D2" s="5">
+        <v>691.88599999999997</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="3" t="s">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="3">
-        <v>283</v>
+      <c r="D3" s="5">
+        <v>654.86200000000008</v>
       </c>
     </row>
   </sheetData>
@@ -510,4 +517,48 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06121D5C-9E82-4DA1-B616-7D25D911AF0F}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="2">
+        <v>299</v>
+      </c>
+      <c r="B1">
+        <f>A1*2.5454</f>
+        <v>761.07459999999992</v>
+      </c>
+      <c r="C1">
+        <f>B1/11</f>
+        <v>69.188599999999994</v>
+      </c>
+      <c r="D1">
+        <f>B1-C1</f>
+        <v>691.88599999999997</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="4">
+        <v>283</v>
+      </c>
+      <c r="B2">
+        <f>A2*2.5454</f>
+        <v>720.34820000000002</v>
+      </c>
+      <c r="C2">
+        <f>B2/11</f>
+        <v>65.486199999999997</v>
+      </c>
+      <c r="D2">
+        <f>B2-C2</f>
+        <v>654.86200000000008</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>